<commit_message>
step4 update figures and PANTHER descriptions
</commit_message>
<xml_diff>
--- a/data/gene_families/manual_annot_panther_families.xlsx
+++ b/data/gene_families/manual_annot_panther_families.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alexis Weinreb\Projects\glia\osc_larva\data\gene_families\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A05A1039-6949-4FCB-A5BD-DE24D473E984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70689F82-EACD-4BCF-81B4-FA103B14E45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{C797D240-5090-4D82-8007-F701C560AE58}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="199">
   <si>
     <t>family</t>
   </si>
@@ -128,9 +128,6 @@
     <t>PTHR24416</t>
   </si>
   <si>
-    <t>description</t>
-  </si>
-  <si>
     <t>cuticlin</t>
   </si>
   <si>
@@ -158,51 +155,21 @@
     <t>glycosyltransferase</t>
   </si>
   <si>
-    <t>nematode astacin metalloprotease</t>
-  </si>
-  <si>
-    <t>cuticle-related</t>
-  </si>
-  <si>
     <t>prion-like</t>
   </si>
   <si>
-    <t>endopeptidase inhibitor</t>
-  </si>
-  <si>
     <t>SXP/RAL-2-like</t>
   </si>
   <si>
     <t>trans thyretin-related</t>
   </si>
   <si>
-    <t>heat-shock protein</t>
-  </si>
-  <si>
-    <t>groundhog-related</t>
-  </si>
-  <si>
-    <t>metallocarboxypeptidase, predicted role in proteolysis</t>
-  </si>
-  <si>
-    <t>domain of unknown function DB</t>
-  </si>
-  <si>
-    <t>unknown</t>
-  </si>
-  <si>
     <t>patched-related</t>
   </si>
   <si>
     <t>receptor tyrosine kinase</t>
   </si>
   <si>
-    <t>nematode-specific peptide family B 7-12</t>
-  </si>
-  <si>
-    <t>nematode-specific peptide family B 1-6</t>
-  </si>
-  <si>
     <t>PTHR22989:SF7</t>
   </si>
   <si>
@@ -281,15 +248,9 @@
     <t>bestrophin</t>
   </si>
   <si>
-    <t>elo acytransferase</t>
-  </si>
-  <si>
     <t>galectin</t>
   </si>
   <si>
-    <t>chaperonin containing TCP-1</t>
-  </si>
-  <si>
     <t>tyrosinase-like</t>
   </si>
   <si>
@@ -311,30 +272,15 @@
     <t>RING domain</t>
   </si>
   <si>
-    <t>SNA-related</t>
-  </si>
-  <si>
-    <t>CUB2 domain</t>
-  </si>
-  <si>
     <t>GOLD domain</t>
   </si>
   <si>
-    <t>proteasome regulatory subunit</t>
-  </si>
-  <si>
     <t>kinesin-like</t>
   </si>
   <si>
     <t>lipase-related</t>
   </si>
   <si>
-    <t>nematode-specific peptide family</t>
-  </si>
-  <si>
-    <t>nhr</t>
-  </si>
-  <si>
     <t>glucuronosyltransferase</t>
   </si>
   <si>
@@ -363,6 +309,330 @@
   </si>
   <si>
     <t>BPI-related</t>
+  </si>
+  <si>
+    <t>astacin metalloprotease</t>
+  </si>
+  <si>
+    <t>metallocarboxypeptidase</t>
+  </si>
+  <si>
+    <t>nsp family B1-6</t>
+  </si>
+  <si>
+    <t>nematode-specific peptide family, group B</t>
+  </si>
+  <si>
+    <t>nematode-specific peptide family, group G</t>
+  </si>
+  <si>
+    <t>nsp family G</t>
+  </si>
+  <si>
+    <t>nsp family B7-12</t>
+  </si>
+  <si>
+    <t>MCM licensing factor</t>
+  </si>
+  <si>
+    <t>DB domain</t>
+  </si>
+  <si>
+    <t>short_description</t>
+  </si>
+  <si>
+    <t>longer_description</t>
+  </si>
+  <si>
+    <t>nas-1, nas-2, …nas-39, hch-1, dpy-31</t>
+  </si>
+  <si>
+    <t>nstp-1, …, nstp-8, ugtp-1, srf-3</t>
+  </si>
+  <si>
+    <t>UDP-sugar transporter</t>
+  </si>
+  <si>
+    <t>BPI2 domain, BPI1 domain, BPI fold-containing protein</t>
+  </si>
+  <si>
+    <t>nrf-5, C55C3.1, C06E8.5</t>
+  </si>
+  <si>
+    <t>best-1, best-2, …</t>
+  </si>
+  <si>
+    <t>ptr-1, ptr-2, …, daf-6</t>
+  </si>
+  <si>
+    <t>Patched-related, SSD domain-containing protein</t>
+  </si>
+  <si>
+    <t>Putative fatty acid elongation protein, Elongation of long chain fatty acids protein</t>
+  </si>
+  <si>
+    <t>elo-1, elo-2, …</t>
+  </si>
+  <si>
+    <t>fatty acid elongation</t>
+  </si>
+  <si>
+    <t>lec-1, lec-2, …</t>
+  </si>
+  <si>
+    <t>T-complex protein 1 subunit</t>
+  </si>
+  <si>
+    <t>cct-1, cct-2, …</t>
+  </si>
+  <si>
+    <t>ShKT domain-containing protein, tyrosinase-like protein, Tyrosinase copper-binding domain-containing protein</t>
+  </si>
+  <si>
+    <t>tyr-1, tyr-2, …</t>
+  </si>
+  <si>
+    <t>tba-1, tba-2, tbb-1, …</t>
+  </si>
+  <si>
+    <t>pas-1, pas-2, pbs-1, ...</t>
+  </si>
+  <si>
+    <t>mcm-2, mcm-3, …</t>
+  </si>
+  <si>
+    <t>gly-3, gly-4, …</t>
+  </si>
+  <si>
+    <t>ShKT domain-containing protein, Peptidase M14 carboxypeptidase A domain-containing protein</t>
+  </si>
+  <si>
+    <t>suro-1, Y18H1A.9, T06A4.1</t>
+  </si>
+  <si>
+    <t>inx-1, inx-2, …</t>
+  </si>
+  <si>
+    <t>Post-GPI attachment to proteins factor 2-like, Frag1_DRAM_Sfk1</t>
+  </si>
+  <si>
+    <t>pgap-2, C14B9.3</t>
+  </si>
+  <si>
+    <t>acr-11, lgc-1, eat-2, …</t>
+  </si>
+  <si>
+    <t>tsp-1, tsp-2, …</t>
+  </si>
+  <si>
+    <t>hsp-1, hsp-70, …</t>
+  </si>
+  <si>
+    <t>RING-type, CUB-like domain-containing protein</t>
+  </si>
+  <si>
+    <t>irg-5, dct-17</t>
+  </si>
+  <si>
+    <t>DUF148 domain-containing protein, SXP_RAL-2 family protein</t>
+  </si>
+  <si>
+    <t>srlf-3, srlf-12, …</t>
+  </si>
+  <si>
+    <t>Glycosyltransferase family 92 protein</t>
+  </si>
+  <si>
+    <t>C13A2.5, R07B7.12</t>
+  </si>
+  <si>
+    <t>T23B3.2, txt-9</t>
+  </si>
+  <si>
+    <t>Pmp3-like</t>
+  </si>
+  <si>
+    <t>Proteolipid membrane potential modulator, SN3-related</t>
+  </si>
+  <si>
+    <t>ttr-6, ttr-17, …</t>
+  </si>
+  <si>
+    <t>irg-8, dod-19, dod-20, hpo-6</t>
+  </si>
+  <si>
+    <t>Transmembrane glycoprotein, Downstream Of DAF-16, IgGFc_binding domain-containing protein, CUB_2 domain-containing protein, Hyphal_reg_CWP domain-containing protein</t>
+  </si>
+  <si>
+    <t>TM glycoprotein</t>
+  </si>
+  <si>
+    <t>FIP (Fungus-Induced Protein) Related, Neuropeptide-like protein, Caenorhabditis bacteriocin</t>
+  </si>
+  <si>
+    <t>fipr-1, …, nlp-24, cnc-1, …</t>
+  </si>
+  <si>
+    <t>tmed-1, …, sel-9</t>
+  </si>
+  <si>
+    <t>GOLD (Golgi dynamics) domain-containing protein</t>
+  </si>
+  <si>
+    <t>Chitotriosidase, Carbohydrate sulfotransferase Chst-1-like, Transposase</t>
+  </si>
+  <si>
+    <t>chst-1, F49D11.6</t>
+  </si>
+  <si>
+    <t>ZP domain-containing protein</t>
+  </si>
+  <si>
+    <t>cutl-2, …, cut-1, …</t>
+  </si>
+  <si>
+    <t>Methyltransferase FkbM domain-containing protein</t>
+  </si>
+  <si>
+    <t>C13A2.9, R09H10.2</t>
+  </si>
+  <si>
+    <t>Acyl_transf_3 domain-containing protein, Acyltransferase</t>
+  </si>
+  <si>
+    <t>oac-1, oac-2, …, bus-1</t>
+  </si>
+  <si>
+    <t>26S proteasome regulatory subunit</t>
+  </si>
+  <si>
+    <t>rpt-1, …</t>
+  </si>
+  <si>
+    <t>proteasome regulatory</t>
+  </si>
+  <si>
+    <t>Kinesin-like protein, Kinesin motor domain-containing protein</t>
+  </si>
+  <si>
+    <t>klp-11, …, unc-116, zen-4</t>
+  </si>
+  <si>
+    <t>Protein kinase domain-containing protein</t>
+  </si>
+  <si>
+    <t>kin-15, daf-2, vab-1, ver-3</t>
+  </si>
+  <si>
+    <t>TCP-1 chaperonin</t>
+  </si>
+  <si>
+    <t>abu-1, …, idpp-5, …, pqn-16, …, appg-2</t>
+  </si>
+  <si>
+    <t>Prion-like-(Q_N-rich)-domain-bearing protein, Activated in Blocked Unfolded protein response</t>
+  </si>
+  <si>
+    <t>Ground-like domain-containing protein, Nucleotide-diphospho-sugar transferase domain-containing protein</t>
+  </si>
+  <si>
+    <t>grd-8, grd-9, …</t>
+  </si>
+  <si>
+    <t>Ground domain</t>
+  </si>
+  <si>
+    <t>lips-2, …, fil-1, …</t>
+  </si>
+  <si>
+    <t>SUP-1-like domain, DUF2650, transmembrane proteins</t>
+  </si>
+  <si>
+    <t>sup-1, C08H9.15, F49F1.14</t>
+  </si>
+  <si>
+    <t>CC domain-containing protein, CHiTin Binding domain (ChtBD2) containing</t>
+  </si>
+  <si>
+    <t>CC domain</t>
+  </si>
+  <si>
+    <t>F08D12.3, chtb-3, hpo-26, pqn-74</t>
+  </si>
+  <si>
+    <t>nspg-1, …</t>
+  </si>
+  <si>
+    <t>nspb-7, …</t>
+  </si>
+  <si>
+    <t>cystein-cradle</t>
+  </si>
+  <si>
+    <t>dpy-6, F09F9.2, Y34B4A.10, F33D4.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leucine-rich repeat-containing protein, ELRR (Extracellular Leucine-Rich Repeat), </t>
+  </si>
+  <si>
+    <t>lron-1, …, dma-1, pan-1</t>
+  </si>
+  <si>
+    <t>Heat shock protein, SHSP domain-containing protein</t>
+  </si>
+  <si>
+    <t>hsp-12.3, hsp-16.11, sip-1</t>
+  </si>
+  <si>
+    <t>Hsp20-like</t>
+  </si>
+  <si>
+    <t>Hsp70-like</t>
+  </si>
+  <si>
+    <t>BPTI_Kunitz inhibitor domain-containing protein, cystein repeat</t>
+  </si>
+  <si>
+    <t>ZC504.1, E01G6.1, K10D3.4</t>
+  </si>
+  <si>
+    <t>CC &amp; Kunitz domains</t>
+  </si>
+  <si>
+    <t>Nuclear Hormone Receptor</t>
+  </si>
+  <si>
+    <t>nhr-73, nhr-251, …</t>
+  </si>
+  <si>
+    <t>DB domain (12 cysteines)</t>
+  </si>
+  <si>
+    <t>C42D4.3, F26G1.5</t>
+  </si>
+  <si>
+    <t>hedgehog-related</t>
+  </si>
+  <si>
+    <t>Ground-like domain-containing protein, Warthog, HintN domain-containing protein</t>
+  </si>
+  <si>
+    <t>qua-1, hog-1, wrt-1, … grd-1, …</t>
+  </si>
+  <si>
+    <t>PAN domain protein, Apple domain-containing protein</t>
+  </si>
+  <si>
+    <t>cutl-17, cutl-27, …, dyf-7, noah-1</t>
+  </si>
+  <si>
+    <t>ugt-2, ugt-12, …</t>
+  </si>
+  <si>
+    <t>UDP-glucuronosyltransferase</t>
+  </si>
+  <si>
+    <t>example_genes</t>
   </si>
 </sst>
 </file>
@@ -734,474 +1004,750 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8CE4E1E-7BFD-4981-9E52-4673D4DD1775}">
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="73.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+      <c r="C1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+      <c r="D2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+      <c r="C3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+      <c r="C4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+      <c r="D5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="C6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="B7" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="C7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C9" t="s">
+        <v>114</v>
+      </c>
+      <c r="D9" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" t="s">
+        <v>116</v>
+      </c>
+      <c r="D10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="B11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B10" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>100</v>
-      </c>
-      <c r="B11" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>77</v>
-      </c>
-      <c r="B13" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>101</v>
-      </c>
       <c r="B14" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="C14" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+      <c r="C15" t="s">
+        <v>122</v>
+      </c>
+      <c r="D15" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="B16" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+      <c r="D16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>7</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+      <c r="C17" t="s">
+        <v>125</v>
+      </c>
+      <c r="D17" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B18" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="D18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="B19" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="D19" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+        <v>183</v>
+      </c>
+      <c r="D20" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="B21" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+      <c r="C21" t="s">
+        <v>130</v>
+      </c>
+      <c r="D21" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>18</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="C22" t="s">
+        <v>132</v>
+      </c>
+      <c r="D22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="C23" t="s">
+        <v>134</v>
+      </c>
+      <c r="D23" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="B24" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+      <c r="C24" t="s">
+        <v>138</v>
+      </c>
+      <c r="D24" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>19</v>
       </c>
       <c r="B25" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="D25" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="B26" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="C26" t="s">
+        <v>141</v>
+      </c>
+      <c r="D26" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>8</v>
       </c>
       <c r="B27" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="C27" t="s">
+        <v>143</v>
+      </c>
+      <c r="D27" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B29" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="C29" t="s">
+        <v>146</v>
+      </c>
+      <c r="D29" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>4</v>
       </c>
       <c r="B30" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="C30" t="s">
+        <v>147</v>
+      </c>
+      <c r="D30" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>1</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+      <c r="C31" t="s">
+        <v>149</v>
+      </c>
+      <c r="D31" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>2</v>
       </c>
       <c r="B32" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+      <c r="C32" t="s">
+        <v>151</v>
+      </c>
+      <c r="D32" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>9</v>
       </c>
       <c r="B34" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+      <c r="C34" t="s">
+        <v>153</v>
+      </c>
+      <c r="D34" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="B35" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+      <c r="C35" t="s">
+        <v>155</v>
+      </c>
+      <c r="D35" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B36" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+      <c r="C36" t="s">
+        <v>158</v>
+      </c>
+      <c r="D36" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="C37" t="s">
+        <v>160</v>
+      </c>
+      <c r="D37" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>5</v>
       </c>
       <c r="B38" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>20</v>
       </c>
       <c r="B39" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+      <c r="C39" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>21</v>
       </c>
       <c r="B40" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+      <c r="C40" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>14</v>
       </c>
       <c r="B41" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="C41" t="s">
+        <v>164</v>
+      </c>
+      <c r="D41" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B42" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+      <c r="C42" t="s">
+        <v>165</v>
+      </c>
+      <c r="D42" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B43" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="D43" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="B44" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+        <v>89</v>
+      </c>
+      <c r="C44" t="s">
+        <v>169</v>
+      </c>
+      <c r="D44" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>12</v>
       </c>
       <c r="B45" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+      <c r="C45" t="s">
+        <v>171</v>
+      </c>
+      <c r="D45" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="B46" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="C46" t="s">
+        <v>95</v>
+      </c>
+      <c r="D46" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>15</v>
       </c>
       <c r="B47" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+      <c r="C47" t="s">
+        <v>94</v>
+      </c>
+      <c r="D47" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>16</v>
       </c>
       <c r="B48" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>27</v>
       </c>
       <c r="B49" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+        <v>176</v>
+      </c>
+      <c r="D49" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="B50" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+      <c r="C50" t="s">
+        <v>178</v>
+      </c>
+      <c r="D50" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>22</v>
       </c>
       <c r="B51" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+        <v>182</v>
+      </c>
+      <c r="C51" t="s">
+        <v>180</v>
+      </c>
+      <c r="D51" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>17</v>
       </c>
       <c r="B52" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+        <v>186</v>
+      </c>
+      <c r="C52" t="s">
+        <v>184</v>
+      </c>
+      <c r="D52" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="B53" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+      <c r="D53" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>25</v>
       </c>
       <c r="B54" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="C54" t="s">
+        <v>189</v>
+      </c>
+      <c r="D54" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>23</v>
       </c>
       <c r="B55" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+      <c r="C55" t="s">
+        <v>192</v>
+      </c>
+      <c r="D55" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>26</v>
       </c>
       <c r="B56" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>3</v>
       </c>
       <c r="B57" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+      <c r="C57" t="s">
+        <v>194</v>
+      </c>
+      <c r="D57" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="B58" t="s">
-        <v>99</v>
+        <v>81</v>
+      </c>
+      <c r="C58" t="s">
+        <v>197</v>
+      </c>
+      <c r="D58" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>